<commit_message>
Adding new BRD for IoT and LoRaWAN capstone project
</commit_message>
<xml_diff>
--- a/history/projects/hsrkom-2024_Capstone-SemesterGenap-TA202324.xlsx
+++ b/history/projects/hsrkom-2024_Capstone-SemesterGenap-TA202324.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10413"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10511"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hsrkom/Documents/__LECTURE NOTES/LNCS_KOM1403_Capstone_Agromaritim40/ilkom-2024_Capstone-K4_03-04/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hsrkom/devsecops/htdocs/office/ilkom/ilkom_isurf/history/projects/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA5A06A5-AFAD-5A40-9336-19ED7B719E0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAD48E2B-D1C0-2142-9013-0F22EF0D7DFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13060" yWindow="2580" windowWidth="26440" windowHeight="15440" xr2:uid="{308D0014-DCB0-D34F-90DE-AC6E12CEEF23}"/>
+    <workbookView xWindow="11960" yWindow="2580" windowWidth="26440" windowHeight="15440" xr2:uid="{308D0014-DCB0-D34F-90DE-AC6E12CEEF23}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Capstone_K4-03_K4-04" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>

</xml_diff>